<commit_message>
Here I go refactoring again
</commit_message>
<xml_diff>
--- a/WorkBot/refactor-experimental/data/order_archive/DUTCH VALLEY FOOD DIST/DUTCH VALLEY FOOD DIST_Bakery_20260216.xlsx
+++ b/WorkBot/refactor-experimental/data/order_archive/DUTCH VALLEY FOOD DIST/DUTCH VALLEY FOOD DIST_Bakery_20260216.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -464,6 +464,258 @@
         <v>48.18</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>832400</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Register Tape - Thermal (3.125" x 230')</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D3" t="n">
+        <v>49.99</v>
+      </c>
+      <c r="E3" t="n">
+        <v>149.97</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>340091</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Raisins - Midget</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" t="n">
+        <v>58.8</v>
+      </c>
+      <c r="E4" t="n">
+        <v>117.6</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>296075</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Nuts - Walnut Halves &amp; Pieces</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D5" t="n">
+        <v>80.98</v>
+      </c>
+      <c r="E5" t="n">
+        <v>242.94</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>384097</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Oats</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>24.84</v>
+      </c>
+      <c r="E6" t="n">
+        <v>24.84</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>462105</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Joe Tea - Classic Lemonade</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="n">
+        <v>22.49</v>
+      </c>
+      <c r="E7" t="n">
+        <v>22.49</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>248058</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Shortening - All Purpose (Palm)</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>4</v>
+      </c>
+      <c r="D8" t="n">
+        <v>69.81</v>
+      </c>
+      <c r="E8" t="n">
+        <v>279.24</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>220252</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Chocolate Block - Bronze Medal</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="n">
+        <v>325.12</v>
+      </c>
+      <c r="E9" t="n">
+        <v>325.12</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>116025</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Sugar - 10X (Powdered)</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" t="n">
+        <v>38.93</v>
+      </c>
+      <c r="E10" t="n">
+        <v>77.86</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>053387</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>DV - Very Berry Pretzels</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="n">
+        <v>36.4</v>
+      </c>
+      <c r="E11" t="n">
+        <v>36.4</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>053125</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>DV - Sour Neon Gummi Worms</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="E12" t="n">
+        <v>32.5</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>053100</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>DV - Gummi Peach Rings</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" t="n">
+        <v>31.04</v>
+      </c>
+      <c r="E13" t="n">
+        <v>31.04</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>456090</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Employee Water</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>20</v>
+      </c>
+      <c r="D14" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="E14" t="n">
+        <v>58.6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>